<commit_message>
Data: Reentrenamiento de modelos Spain + Collect_predictions.py de todas las ligas
</commit_message>
<xml_diff>
--- a/p2_data_understanding/data/spain/df_teams_sofifa.xlsx
+++ b/p2_data_understanding/data/spain/df_teams_sofifa.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,22 +473,22 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>452</t>
+          <t>243</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Espanyol</t>
+          <t>Real Madrid</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>RCDE Stadium</t>
+          <t>Estadio Santiago Bernabéu</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -508,7 +508,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://sofifa.com/team/452/espanyol/</t>
+          <t>https://sofifa.com/team/243/real-madrid/</t>
         </is>
       </c>
       <c r="I2" t="n">
@@ -518,42 +518,42 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>462</t>
+          <t>241</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Real Valladolid</t>
+          <t>FC Barcelona</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Estadio José Zorrilla</t>
+          <t>El Libertador</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>459</t>
+          <t>243</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Sporting Gijón</t>
+          <t>Real Madrid</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://sofifa.com/team/462/real-valladolid/</t>
+          <t>https://sofifa.com/team/241/fc-barcelona/</t>
         </is>
       </c>
       <c r="I3" t="n">
@@ -563,22 +563,22 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>1853</t>
+          <t>240</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Levante</t>
+          <t>Atlético Madrid</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Estadio Ciutat de València</t>
+          <t>Wanda Metropolitano</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -588,17 +588,17 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>461</t>
+          <t>243</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Valencia</t>
+          <t>Real Madrid</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://sofifa.com/team/1853/levante/</t>
+          <t>https://sofifa.com/team/240/atletico-madrid/</t>
         </is>
       </c>
       <c r="I4" t="n">
@@ -608,22 +608,22 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>459</t>
+          <t>448</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Sporting Gijón</t>
+          <t>Athletic Club</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Stade Municipal</t>
+          <t>Estadio San Mamés</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>110827</t>
+          <t>457</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Real Oviedo</t>
+          <t>Real Sociedad</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://sofifa.com/team/459/sporting-gijon/</t>
+          <t>https://sofifa.com/team/448/athletic-club/</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -653,42 +653,42 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>467</t>
+          <t>457</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>SD Eibar</t>
+          <t>Real Sociedad</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Municipal de Ipurua</t>
+          <t>Reale Arena</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>457</t>
+          <t>448</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Real Sociedad</t>
+          <t>Athletic Club</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://sofifa.com/team/467/sd-eibar/</t>
+          <t>https://sofifa.com/team/457/real-sociedad/</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -698,42 +698,42 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>110827</t>
+          <t>481</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Real Oviedo</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Stadion Europa</t>
+          <t>Ramón Sánchez-Pizjuán</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>459</t>
+          <t>449</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Sporting Gijón</t>
+          <t>Real Betis</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://sofifa.com/team/110827/real-oviedo/</t>
+          <t>https://sofifa.com/team/481/sevilla/</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -743,42 +743,42 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>244</t>
+          <t>110062</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Real Zaragoza</t>
+          <t>Girona</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>El Libertador</t>
+          <t>Estadio de Montilivi</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>110839</t>
+          <t>452</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Huesca</t>
+          <t>Espanyol</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://sofifa.com/team/244/real-zaragoza/</t>
+          <t>https://sofifa.com/team/110062/girona/</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -788,42 +788,42 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>449</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Tenerife</t>
+          <t>Real Betis</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Stadio Classico</t>
+          <t>Estadio Benito Villamarín</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>472</t>
+          <t>481</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Las Palmas</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://sofifa.com/team/260/tenerife/</t>
+          <t>https://sofifa.com/team/449/real-betis/</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -833,42 +833,42 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>100888</t>
+          <t>483</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Leganés</t>
+          <t>Villarreal</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Municipal de Butarque</t>
+          <t>Estadio de la Cerámica</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>1860</t>
+          <t>461</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Getafe</t>
+          <t>Valencia</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://sofifa.com/team/100888/leganes/</t>
+          <t>https://sofifa.com/team/483/villarreal/</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -878,42 +878,42 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>10846</t>
+          <t>1860</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Burgos</t>
+          <t>Getafe</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Court Lane</t>
+          <t>Coliseum Alfonso Pérez</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>110069</t>
+          <t>100888</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Mirandés</t>
+          <t>Leganés</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://sofifa.com/team/10846/burgos/</t>
+          <t>https://sofifa.com/team/1860/getafe/</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -923,42 +923,42 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>468</t>
+          <t>450</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Elche</t>
+          <t>Celta de Vigo</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Estadio Martínez Valero</t>
+          <t>Estadio Abanca-Balaídos</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1853</t>
+          <t>110242</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Levante</t>
+          <t>Racing Ferrol</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://sofifa.com/team/468/elche/</t>
+          <t>https://sofifa.com/team/450/celta-de-vigo/</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -968,17 +968,17 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>1854</t>
+          <t>453</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Albacete</t>
+          <t>Mallorca</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Estadio Nacional</t>
+          <t>Visit Mallorca Estadi</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -988,22 +988,22 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1853</t>
+          <t>483</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Levante</t>
+          <t>Villarreal</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://sofifa.com/team/1854/albacete/</t>
+          <t>https://sofifa.com/team/453/mallorca/</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -1013,17 +1013,17 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>456</t>
+          <t>479</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Racing Santander</t>
+          <t>Osasuna</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Stade Municipal</t>
+          <t>Estadio El Sadar</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://sofifa.com/team/456/racing-santander/</t>
+          <t>https://sofifa.com/team/479/osasuna/</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -1058,17 +1058,17 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>110839</t>
+          <t>480</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Huesca</t>
+          <t>Rayo Vallecano</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>El Alcoraz</t>
+          <t>Estadio de Vallecas</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1078,22 +1078,22 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>244</t>
+          <t>100888</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Real Zaragoza</t>
+          <t>Leganés</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://sofifa.com/team/110839/huesca/</t>
+          <t>https://sofifa.com/team/480/rayo-vallecano/</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -1103,17 +1103,17 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>131110</t>
+          <t>1861</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Eldense</t>
+          <t>Almería</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Town Park</t>
+          <t>Power Horse Stadium</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1123,22 +1123,22 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>468</t>
+          <t>110832</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Elche</t>
+          <t>Granada</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://sofifa.com/team/131110/eldense/</t>
+          <t>https://sofifa.com/team/1861/almeria/</t>
         </is>
       </c>
       <c r="I16" t="n">
@@ -1148,17 +1148,17 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>110242</t>
+          <t>1968</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Racing Ferrol</t>
+          <t>Cádiz</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Town Park</t>
+          <t>Nuevo Mirandilla</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1168,22 +1168,22 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>450</t>
+          <t>481</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Celta de Vigo</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://sofifa.com/team/110242/racing-ferrol/</t>
+          <t>https://sofifa.com/team/1968/cadiz/</t>
         </is>
       </c>
       <c r="I17" t="n">
@@ -1193,27 +1193,27 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>110902</t>
+          <t>461</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Villarreal II</t>
+          <t>Valencia</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Estadio de la Cerámica</t>
+          <t>Estadio Mestalla</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1228,7 +1228,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://sofifa.com/team/110902/villarreal-ii/</t>
+          <t>https://sofifa.com/team/461/valencia/</t>
         </is>
       </c>
       <c r="I18" t="n">
@@ -1238,17 +1238,17 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>114554</t>
+          <t>472</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>FC Andorra</t>
+          <t>Las Palmas</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Town Park</t>
+          <t>Estadio de Gran Canaria</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1258,22 +1258,22 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>110062</t>
+          <t>260</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Girona</t>
+          <t>Tenerife</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://sofifa.com/team/114554/fc-andorra/</t>
+          <t>https://sofifa.com/team/472/las-palmas/</t>
         </is>
       </c>
       <c r="I19" t="n">
@@ -1283,17 +1283,17 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>100831</t>
+          <t>463</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Alcorcón</t>
+          <t>Deportivo Alavés</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Town Park</t>
+          <t>Estadio de Mendizorroza</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1303,22 +1303,22 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>448</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Rayo Vallecano</t>
+          <t>Athletic Club</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://sofifa.com/team/100831/alcorcon/</t>
+          <t>https://sofifa.com/team/463/deportivo-alaves/</t>
         </is>
       </c>
       <c r="I20" t="n">
@@ -1328,17 +1328,17 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>100851</t>
+          <t>110832</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>FC Cartagena</t>
+          <t>Granada</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Stadio Classico</t>
+          <t>Estadio Nuevo Los Cármenes</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1348,22 +1348,22 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>468</t>
+          <t>449</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Elche</t>
+          <t>Real Betis</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://sofifa.com/team/100851/fc-cartagena/</t>
+          <t>https://sofifa.com/team/110832/granada/</t>
         </is>
       </c>
       <c r="I21" t="n">
@@ -1373,42 +1373,42 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>113356</t>
+          <t>452</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Amorebieta</t>
+          <t>Espanyol</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Town Park</t>
+          <t>Stage Front Stadium</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>467</t>
+          <t>241</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>SD Eibar</t>
+          <t>FC Barcelona</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://sofifa.com/team/113356/amorebieta/</t>
+          <t>https://sofifa.com/team/452/espanyol/</t>
         </is>
       </c>
       <c r="I22" t="n">
@@ -1418,45 +1418,945 @@
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
+          <t>100888</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Leganés</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Municipal de Butarque</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>1860</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Getafe</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/100888/leganes/</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>462</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Real Valladolid</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Estadio José Zorrilla</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>459</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Sporting Gijón</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/462/real-valladolid/</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>467</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>SD Eibar</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Municipal de Ipurua</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>457</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Real Sociedad</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/467/sd-eibar/</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>110827</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Real Oviedo</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Stadion Europa</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>459</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Sporting Gijón</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/110827/real-oviedo/</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>260</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Tenerife</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Stadio Classico</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>472</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Las Palmas</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/260/tenerife/</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>1853</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Levante</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Estadio Ciutat de València</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>461</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Valencia</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/1853/levante/</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>459</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Sporting Gijón</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Stade Municipal</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>110827</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Real Oviedo</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/459/sporting-gijon/</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>468</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Elche</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Estadio Martínez Valero</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>1853</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Levante</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/468/elche/</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>244</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Real Zaragoza</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>El Libertador</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>110839</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Huesca</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/244/real-zaragoza/</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="inlineStr">
+        <is>
+          <t>10846</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Burgos</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Court Lane</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
           <t>110069</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="G32" t="inlineStr">
         <is>
           <t>Mirandés</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/10846/burgos/</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="inlineStr">
+        <is>
+          <t>456</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Racing Santander</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Stade Municipal</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>448</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Athletic Club</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/456/racing-santander/</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="inlineStr">
+        <is>
+          <t>110839</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Huesca</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>El Alcoraz</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>244</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Real Zaragoza</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/110839/huesca/</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="inlineStr">
+        <is>
+          <t>131110</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Eldense</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
         <is>
           <t>Town Park</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>468</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Elche</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/131110/eldense/</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="inlineStr">
+        <is>
+          <t>1854</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Albacete</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Estadio Nacional</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>1853</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Levante</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/1854/albacete/</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="inlineStr">
+        <is>
+          <t>110242</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Racing Ferrol</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Town Park</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>450</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Celta de Vigo</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/110242/racing-ferrol/</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="inlineStr">
+        <is>
+          <t>110902</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Villarreal II</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Estadio de la Cerámica</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>1853</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Levante</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/110902/villarreal-ii/</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="inlineStr">
+        <is>
+          <t>114554</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>FC Andorra</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Town Park</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>110062</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Girona</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/114554/fc-andorra/</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="inlineStr">
+        <is>
+          <t>100831</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Alcorcón</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Town Park</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>480</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Rayo Vallecano</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/100831/alcorcon/</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="inlineStr">
+        <is>
+          <t>100851</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>FC Cartagena</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Stadio Classico</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>468</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Elche</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/100851/fc-cartagena/</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="inlineStr">
+        <is>
+          <t>113356</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Amorebieta</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Town Park</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>467</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>SD Eibar</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/113356/amorebieta/</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="inlineStr">
+        <is>
+          <t>110069</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Mirandés</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Town Park</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F43" t="inlineStr">
         <is>
           <t>463</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="G43" t="inlineStr">
         <is>
           <t>Deportivo Alavés</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="H43" t="inlineStr">
         <is>
           <t>https://sofifa.com/team/110069/mirandes/</t>
         </is>
       </c>
-      <c r="I23" t="n">
+      <c r="I43" t="n">
         <v>148</v>
       </c>
     </row>

</xml_diff>